<commit_message>
xlstream-eval: fix bitwise fixture NA() column pollution
B25/B26 had =NA() formulas, causing the template rewriter to treat
column B as a formula column and overwrite data rows with NA().
Moved NA() to column E. Fixed cross-sheet ref in D32 with literal.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/engineering/bitwise.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/engineering/bitwise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_706427580966BBD1984FD1763D1012548D0AC4FB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_15AD0CF9FB2C1AD73068B1B73E3D82177C77CEA2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -481,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -723,7 +723,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -738,7 +738,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -753,7 +753,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -768,7 +768,7 @@
         <v>281474976710655</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -783,7 +783,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -798,7 +798,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -813,7 +813,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -828,7 +828,7 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -843,39 +843,39 @@
         <v>#NUM!</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>27</v>
       </c>
-      <c r="B25" t="e">
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="e">
+        <f>_xlfn.BITAND(E25,C25)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E25" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25" t="e">
-        <f>_xlfn.BITAND(B25,C25)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>28</v>
       </c>
-      <c r="B26" t="e">
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="e">
+        <f>_xlfn.BITLSHIFT(E26,C26)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E26" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
-      <c r="D26" t="e">
-        <f>_xlfn.BITLSHIFT(B26,C26)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -890,7 +890,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -905,7 +905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -920,7 +920,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -935,12 +935,12 @@
         <v>odd</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>34</v>
       </c>
       <c r="D32">
-        <f>_xlfn.BITXOR(Sheet2!A2,Sheet2!A3)</f>
+        <f>_xlfn.BITXOR(13,25)</f>
         <v>20</v>
       </c>
     </row>

</xml_diff>